<commit_message>
SSLC cash check: mark $864K billed-ahead as disputed (John 10/10)
</commit_message>
<xml_diff>
--- a/drafts/SSLC_YearEnd_Cash_Reality_Check_2026-10-10.xlsx
+++ b/drafts/SSLC_YearEnd_Cash_Reality_Check_2026-10-10.xlsx
@@ -801,7 +801,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>SSLC QB 10/2: $864K billed ahead + $120K deposits</t>
+          <t>SSLC QB 10/2: $864K billed ahead + $120K deposits. DISPUTED by John: tank start/billing not captured correctly</t>
         </is>
       </c>
     </row>
@@ -881,7 +881,7 @@
       </c>
       <c r="E1" s="5" t="inlineStr">
         <is>
-          <t>Realistic: cash balance</t>
+          <t>Per SSLC books (disputed): cash balance</t>
         </is>
       </c>
       <c r="F1" s="5" t="inlineStr">
@@ -1359,7 +1359,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Realistic year-end cash (prepaid backlog first)</t>
+          <t>Per SSLC books, if billed-ahead is accurate (DISPUTED)</t>
         </is>
       </c>
       <c r="B6" s="6">
@@ -1392,7 +1392,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Shortfall vs claim: realistic</t>
+          <t>Shortfall vs claim: per SSLC books (disputed)</t>
         </is>
       </c>
       <c r="B9" s="6">

</xml_diff>

<commit_message>
SSLC cash check xlsx: 'per SSLC books, disputed by John Quinn' labels
</commit_message>
<xml_diff>
--- a/drafts/SSLC_YearEnd_Cash_Reality_Check_2026-10-10.xlsx
+++ b/drafts/SSLC_YearEnd_Cash_Reality_Check_2026-10-10.xlsx
@@ -801,7 +801,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>SSLC QB 10/2: $864K billed ahead + $120K deposits. DISPUTED by John: tank start/billing not captured correctly</t>
+          <t>SSLC QB 10/2: $864K billed ahead + $120K deposits. Per SSLC books, disputed by John Quinn — tank start/billing not captured correctly</t>
         </is>
       </c>
     </row>
@@ -881,7 +881,7 @@
       </c>
       <c r="E1" s="5" t="inlineStr">
         <is>
-          <t>Per SSLC books (disputed): cash balance</t>
+          <t>Per SSLC books, disputed by John Quinn: cash balance</t>
         </is>
       </c>
       <c r="F1" s="5" t="inlineStr">
@@ -899,7 +899,6 @@
       <c r="A2" t="n">
         <v>0</v>
       </c>
-      <c r="B2" t="inlineStr"/>
       <c r="C2" s="6" t="n">
         <v>0</v>
       </c>
@@ -1323,6 +1322,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -1359,7 +1359,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Per SSLC books, if billed-ahead is accurate (DISPUTED)</t>
+          <t>Per SSLC books, disputed by John Quinn (if billed-ahead figure is accurate)</t>
         </is>
       </c>
       <c r="B6" s="6">
@@ -1392,7 +1392,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Shortfall vs claim: per SSLC books (disputed)</t>
+          <t>Shortfall vs claim: per SSLC books, disputed by John Quinn</t>
         </is>
       </c>
       <c r="B9" s="6">
@@ -1400,6 +1400,7 @@
         <v/>
       </c>
     </row>
+    <row r="10"/>
     <row r="11" ht="60" customHeight="1">
       <c r="A11" s="8" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
SSLC cash check rebased on 10/11 QB balance sheet ($590K cash, $942K billed ahead)
</commit_message>
<xml_diff>
--- a/drafts/SSLC_YearEnd_Cash_Reality_Check_2026-10-10.xlsx
+++ b/drafts/SSLC_YearEnd_Cash_Reality_Check_2026-10-10.xlsx
@@ -197,12 +197,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Weekly Cash'!$A$2:$A$15</f>
+              <f>'Weekly Cash'!$A$2:$A$14</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Weekly Cash'!$D$2:$D$15</f>
+              <f>'Weekly Cash'!$D$2:$D$14</f>
             </numRef>
           </val>
         </ser>
@@ -229,12 +229,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Weekly Cash'!$A$2:$A$15</f>
+              <f>'Weekly Cash'!$A$2:$A$14</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Weekly Cash'!$E$2:$E$15</f>
+              <f>'Weekly Cash'!$E$2:$E$14</f>
             </numRef>
           </val>
         </ser>
@@ -261,12 +261,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Weekly Cash'!$A$2:$A$15</f>
+              <f>'Weekly Cash'!$A$2:$A$14</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Weekly Cash'!$F$2:$F$15</f>
+              <f>'Weekly Cash'!$F$2:$F$14</f>
             </numRef>
           </val>
         </ser>
@@ -293,12 +293,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Weekly Cash'!$A$2:$A$15</f>
+              <f>'Weekly Cash'!$A$2:$A$14</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Weekly Cash'!$G$2:$G$15</f>
+              <f>'Weekly Cash'!$G$2:$G$14</f>
             </numRef>
           </val>
         </ser>
@@ -320,7 +320,7 @@
                   <a:defRPr/>
                 </a:pPr>
                 <a:r>
-                  <a:t>Week from Oct 2</a:t>
+                  <a:t>Week from Oct 11</a:t>
                 </a:r>
               </a:p>
             </rich>
@@ -718,15 +718,15 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Starting cash (Oct 2, 2026)</t>
+          <t>Starting cash (Oct 11, 2026)</t>
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>198000</v>
+        <v>590344</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>SSLC QuickBooks pull 10/2/2026</t>
+          <t>SSLC QuickBooks Balance Sheet as of 10/11/2026 (John export)</t>
         </is>
       </c>
     </row>
@@ -748,15 +748,15 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Weeks Oct 2 → Dec 31</t>
+          <t>Weeks Oct 11 → Dec 31</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Calendar</t>
+          <t>Calendar (~11.6 weeks)</t>
         </is>
       </c>
     </row>
@@ -797,11 +797,11 @@
         </is>
       </c>
       <c r="B8" s="3" t="n">
-        <v>984000</v>
+        <v>1062177</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>SSLC QB 10/2: $864K billed ahead + $120K deposits. Per SSLC books, disputed by John Quinn — tank start/billing not captured correctly</t>
+          <t>SSLC QB 10/11: $942,177 billed ahead (AR Unbilled) + $120K deposits. DISPUTED by John: tank start/billing not captured correctly</t>
         </is>
       </c>
     </row>
@@ -846,7 +846,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G15"/>
+  <dimension ref="A1:G14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -881,7 +881,7 @@
       </c>
       <c r="E1" s="5" t="inlineStr">
         <is>
-          <t>Per SSLC books, disputed by John Quinn: cash balance</t>
+          <t>Per SSLC books (disputed): cash balance</t>
         </is>
       </c>
       <c r="F1" s="5" t="inlineStr">
@@ -899,6 +899,7 @@
       <c r="A2" t="n">
         <v>0</v>
       </c>
+      <c r="B2" t="inlineStr"/>
       <c r="C2" s="6" t="n">
         <v>0</v>
       </c>
@@ -1263,35 +1264,6 @@
         <v/>
       </c>
       <c r="G14" s="6">
-        <f>Inputs!$B$4</f>
-        <v/>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="n">
-        <v>13</v>
-      </c>
-      <c r="B15">
-        <f>IF(MOD(A15,Inputs!$B$6)=0,"Yes","")</f>
-        <v/>
-      </c>
-      <c r="C15" s="6">
-        <f>IF(B15="Yes",Inputs!$B$7,0)</f>
-        <v/>
-      </c>
-      <c r="D15" s="6">
-        <f>D14+C15-Inputs!$B$7*Inputs!$B$9/Inputs!$B$6-Inputs!$B$10/52</f>
-        <v/>
-      </c>
-      <c r="E15" s="6">
-        <f>E14+MAX(0,SUM($C$3:C15)-Inputs!$B$8)-MAX(0,SUM($C$3:C14)-Inputs!$B$8)-Inputs!$B$7*Inputs!$B$9/Inputs!$B$6-Inputs!$B$10/52</f>
-        <v/>
-      </c>
-      <c r="F15" s="6">
-        <f>Inputs!$B$3+(Inputs!$B$4-Inputs!$B$3)*A15/Inputs!$B$5</f>
-        <v/>
-      </c>
-      <c r="G15" s="6">
         <f>Inputs!$B$4</f>
         <v/>
       </c>
@@ -1322,7 +1294,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -1330,7 +1301,7 @@
         </is>
       </c>
       <c r="B3" s="7">
-        <f>COUNTIF('Weekly Cash'!B3:B15,"Yes")</f>
+        <f>COUNTIF('Weekly Cash'!B3:B14,"Yes")</f>
         <v/>
       </c>
     </row>
@@ -1341,7 +1312,7 @@
         </is>
       </c>
       <c r="B4" s="6">
-        <f>SUM('Weekly Cash'!C3:C15)</f>
+        <f>SUM('Weekly Cash'!C3:C14)</f>
         <v/>
       </c>
     </row>
@@ -1352,18 +1323,18 @@
         </is>
       </c>
       <c r="B5" s="6">
-        <f>'Weekly Cash'!D15</f>
+        <f>'Weekly Cash'!D14</f>
         <v/>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Per SSLC books, disputed by John Quinn (if billed-ahead figure is accurate)</t>
+          <t>Per SSLC books, if billed-ahead is accurate (DISPUTED)</t>
         </is>
       </c>
       <c r="B6" s="6">
-        <f>'Weekly Cash'!E15</f>
+        <f>'Weekly Cash'!E14</f>
         <v/>
       </c>
     </row>
@@ -1392,7 +1363,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Shortfall vs claim: per SSLC books, disputed by John Quinn</t>
+          <t>Shortfall vs claim: per SSLC books (disputed)</t>
         </is>
       </c>
       <c r="B9" s="6">
@@ -1400,11 +1371,10 @@
         <v/>
       </c>
     </row>
-    <row r="10"/>
     <row r="11" ht="60" customHeight="1">
       <c r="A11" s="8" t="inlineStr">
         <is>
-          <t>Reading: even if every tank is new cash, SSLC can't reach $850K by year-end from operations. The prepaid backlog means the next ~4 tanks were already paid for. Reaching $850K requires new customer deposits or financing, and each of those adds a delivery or repayment obligation.</t>
+          <t>Reading: SSLC held $590K on 10/11 (up from $198K on 10/2), mostly from collecting receivables and billing ahead: the billed-ahead balance is $942K and still rising. Even if every tank from here is new cash, year-end lands near the claim only in the best case. If the billed-ahead work is owed as booked, finishing it drains cash below zero. Either way the cash reflects customer prepayment, not earnings.</t>
         </is>
       </c>
     </row>

</xml_diff>